<commit_message>
Working but failing on recursion due to client error?
</commit_message>
<xml_diff>
--- a/wis2box/oregon/xlsx/tests/IoW_Reccomended_Obs_Data_Elements.xlsx
+++ b/wis2box/oregon/xlsx/tests/IoW_Reccomended_Obs_Data_Elements.xlsx
@@ -9,6 +9,11 @@
   </sheets>
   <definedNames/>
   <calcPr/>
+  <extLst>
+    <ext uri="GoogleSheetsCustomDataVersion2">
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="yrNMqY0116cGJKiR0EWkP2uwSmCREQk4crusYJ83YO0="/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -45,7 +50,7 @@
     <t>Feature of Interest Name</t>
   </si>
   <si>
-    <t>Feature of Interest  URI</t>
+    <t>Feature of Interest URI</t>
   </si>
   <si>
     <t>River Site A</t>
@@ -312,7 +317,6 @@
     <font>
       <color theme="1"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -353,7 +357,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -365,14 +369,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="top"/>
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -599,7 +598,6 @@
     <col customWidth="1" min="5" max="5" width="31.29"/>
     <col customWidth="1" min="6" max="8" width="16.29"/>
     <col customWidth="1" min="9" max="11" width="26.43"/>
-    <col customWidth="1" min="12" max="26" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -627,10 +625,10 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="2" t="s">
@@ -662,13 +660,13 @@
       <c r="H2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="5" t="s">
         <v>21</v>
       </c>
     </row>
@@ -700,10 +698,10 @@
       <c r="I3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="K3" s="5" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1710,11 +1708,11 @@
   <cols>
     <col customWidth="1" min="1" max="3" width="29.57"/>
     <col customWidth="1" min="4" max="4" width="41.57"/>
-    <col customWidth="1" min="5" max="27" width="29.57"/>
+    <col customWidth="1" min="5" max="15" width="29.57"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>33</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -2859,7 +2857,12 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="26" width="8.71"/>
+    <col customWidth="1" min="1" max="1" width="8.71"/>
+    <col customWidth="1" min="2" max="2" width="27.86"/>
+    <col customWidth="1" min="3" max="3" width="24.0"/>
+    <col customWidth="1" min="4" max="4" width="17.57"/>
+    <col customWidth="1" min="5" max="5" width="25.43"/>
+    <col customWidth="1" min="6" max="6" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>